<commit_message>
added excel export support for vendors/customers and organizations
</commit_message>
<xml_diff>
--- a/src/templates/processed-purchase-invoices-template.xlsx
+++ b/src/templates/processed-purchase-invoices-template.xlsx
@@ -375,14 +375,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:BF3"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:BF2"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14.35"/>
@@ -393,22 +393,22 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="21.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="24.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="12.41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="14.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="14.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="12.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="24.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="20.18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="21.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="19.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="19.2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="17.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="15.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="17.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="18.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="17.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="18.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="18.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="16.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="23.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="23.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="13.93"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="20.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="24.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="24.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="0" width="14.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="0" width="16.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="17.13"/>
@@ -422,13 +422,13 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="0" width="10.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="0" width="12.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="0" width="12.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="48" style="0" width="25.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="48" style="0" width="25.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="49" min="49" style="0" width="29.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="50" min="50" style="0" width="17.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="51" min="51" style="0" width="25.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="52" min="52" style="0" width="18.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="52" min="52" style="0" width="18.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="53" min="53" style="0" width="25.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="54" min="54" style="0" width="18.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="54" min="54" style="0" width="18.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="55" min="55" style="0" width="24.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="56" min="56" style="0" width="18.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="57" min="57" style="0" width="23.8"/>
@@ -669,66 +669,6 @@
       <c r="BE2" s="2"/>
       <c r="BF2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
-      <c r="W3" s="2"/>
-      <c r="X3" s="2"/>
-      <c r="Y3" s="2"/>
-      <c r="Z3" s="2"/>
-      <c r="AA3" s="2"/>
-      <c r="AB3" s="2"/>
-      <c r="AC3" s="2"/>
-      <c r="AD3" s="2"/>
-      <c r="AE3" s="2"/>
-      <c r="AF3" s="2"/>
-      <c r="AG3" s="2"/>
-      <c r="AH3" s="2"/>
-      <c r="AI3" s="2"/>
-      <c r="AJ3" s="2"/>
-      <c r="AK3" s="2"/>
-      <c r="AL3" s="2"/>
-      <c r="AM3" s="2"/>
-      <c r="AN3" s="2"/>
-      <c r="AO3" s="2"/>
-      <c r="AP3" s="2"/>
-      <c r="AQ3" s="2"/>
-      <c r="AR3" s="2"/>
-      <c r="AS3" s="2"/>
-      <c r="AT3" s="2"/>
-      <c r="AU3" s="2"/>
-      <c r="AV3" s="2"/>
-      <c r="AW3" s="2"/>
-      <c r="AX3" s="2"/>
-      <c r="AY3" s="2"/>
-      <c r="AZ3" s="2"/>
-      <c r="BA3" s="2"/>
-      <c r="BB3" s="2"/>
-      <c r="BC3" s="2"/>
-      <c r="BD3" s="2"/>
-      <c r="BE3" s="2"/>
-      <c r="BF3" s="2"/>
-    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>